<commit_message>
modify nominal pipe size
</commit_message>
<xml_diff>
--- a/tests/input/2604081338_Sample-Class-Input/Class_Define_Template.xlsx
+++ b/tests/input/2604081338_Sample-Class-Input/Class_Define_Template.xlsx
@@ -6,22 +6,23 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="510" yWindow="600" windowWidth="27735" windowHeight="11700" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Class_Define" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Fluid_Service" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Joint" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Schedule" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Branch_Table" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Reducing_Table" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Pipe_Group" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Fitting_Group" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Flange_Group" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Gasket_Group" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Valve" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Unit_System" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Class_Define" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Fluid_Service" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Joint" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Schedule" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Branch_Table" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Reducing_Table" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Pipe_Group" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Fitting_Group" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Flange_Group" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Gasket_Group" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Valve" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Branch_Table'!$A$1:$E$125</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Reducing_Table'!$A$1:$E$56</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Fitting_Group'!$A$1:$L$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Branch_Table'!$A$1:$E$125</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Reducing_Table'!$A$1:$E$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Fitting_Group'!$A$1:$L$27</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -30,7 +31,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="맑은 고딕"/>
       <family val="2"/>
@@ -52,8 +53,11 @@
       <sz val="8"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -64,6 +68,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -79,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -88,6 +98,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -455,143 +468,228 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Unit_System</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Design_Temperature_Unit</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Design_Pressure_Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>°C</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
-    <col width="13" customWidth="1" style="3" min="1" max="1"/>
-    <col width="12" customWidth="1" style="3" min="2" max="2"/>
-    <col width="13" customWidth="1" style="3" min="3" max="3"/>
-    <col width="21" customWidth="1" style="3" min="4" max="4"/>
-    <col width="14" customWidth="1" style="3" min="5" max="5"/>
-    <col width="21" customWidth="1" style="3" min="6" max="6"/>
-    <col width="25" customWidth="1" style="3" min="7" max="7"/>
-    <col width="23" customWidth="1" style="3" min="8" max="8"/>
-    <col width="22" customWidth="1" style="3" min="9" max="9"/>
-    <col width="20" customWidth="1" style="3" min="10" max="10"/>
-    <col width="15" customWidth="1" style="3" min="11" max="11"/>
-    <col width="16" customWidth="1" style="3" min="12" max="13"/>
-    <col width="18" customWidth="1" style="3" min="14" max="15"/>
-    <col width="20" customWidth="1" style="3" min="16" max="16"/>
-    <col width="12" customWidth="1" style="3" min="17" max="17"/>
-    <col width="9" customWidth="1" style="3" min="18" max="16384"/>
+    <col width="12" customWidth="1" style="3" min="1" max="10"/>
+    <col width="13" customWidth="1" style="3" min="11" max="11"/>
+    <col width="14" customWidth="1" style="3" min="12" max="12"/>
+    <col width="12" customWidth="1" style="3" min="13" max="13"/>
+    <col width="9" customWidth="1" style="3" min="14" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Revision_No</t>
+          <t>Class_Name</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Class_Name</t>
+          <t>Item_Code</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Design_Code</t>
+          <t>Size1_From</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Class_Base_Material</t>
+          <t>Size1_To</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Class_Rating</t>
+          <t>Size2_From</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Corrosion_Allowance</t>
+          <t>Size2_To</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Design_Temperature_From [°C]</t>
+          <t>Mat_Code</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Design_Temperature_To [°C]</t>
+          <t>Mat_Class</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Design_Pressure_From [bar]</t>
+          <t>Rating</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Design_Pressure_To [bar]</t>
+          <t>Facing</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Fluid_Service</t>
+          <t>Flange_Type</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Branch_Table_1</t>
+          <t>Dim_Standard</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Branch_Table_2</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Reducing_Table_1</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Reducing_Table_2</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Global_Special_Req</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
           <t>Remarks</t>
         </is>
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>AA1</t>
+        </is>
+      </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>A105</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>CL150</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>RF</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>SW</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>ASME B16.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
           <t>AA1</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>KCS</t>
-        </is>
-      </c>
-      <c r="L2" s="3" t="inlineStr">
-        <is>
-          <t>BT1</t>
-        </is>
-      </c>
-      <c r="N2" s="3" t="inlineStr">
-        <is>
-          <t>RT1</t>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>A105</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>CL150</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>RF</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>WN</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>ASME B16.5</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -757,7 +855,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -857,6 +955,163 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:R2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
+  <cols>
+    <col width="13" customWidth="1" style="3" min="1" max="1"/>
+    <col width="12" customWidth="1" style="3" min="2" max="2"/>
+    <col width="13" customWidth="1" style="3" min="3" max="3"/>
+    <col width="21" customWidth="1" style="3" min="4" max="4"/>
+    <col width="14" customWidth="1" style="3" min="5" max="5"/>
+    <col width="21" customWidth="1" style="3" min="6" max="6"/>
+    <col width="25" customWidth="1" style="3" min="7" max="7"/>
+    <col width="23" customWidth="1" style="3" min="8" max="8"/>
+    <col width="22" customWidth="1" style="3" min="9" max="9"/>
+    <col width="20" customWidth="1" style="3" min="10" max="10"/>
+    <col width="15" customWidth="1" style="3" min="11" max="11"/>
+    <col width="16" customWidth="1" style="3" min="12" max="13"/>
+    <col width="18" customWidth="1" style="3" min="14" max="15"/>
+    <col width="20" customWidth="1" style="3" min="16" max="16"/>
+    <col width="12" customWidth="1" style="3" min="17" max="17"/>
+    <col width="9" customWidth="1" style="3" min="18" max="16384"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Revision_No</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Class_Name</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Nominal_Size_System</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Design_Code</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Class_Base_Material</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Class_Rating</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Corrosion_Allowance</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Design_Temperature_From [°C]</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Design_Temperature_To [°C]</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Design_Pressure_From [bar]</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Design_Pressure_To [bar]</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Fluid_Service</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Branch_Table_1</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Branch_Table_2</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Reducing_Table_1</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Reducing_Table_2</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Global_Special_Req</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>AA1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ASME B31.3</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>KCS</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>BT1</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>RT1</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
@@ -920,7 +1175,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -973,7 +1228,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1067,7 +1322,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3841,7 +4096,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5097,7 +5352,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5492,7 +5747,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6851,178 +7106,4 @@
   <autoFilter ref="A1:L27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
-  <cols>
-    <col width="12" customWidth="1" style="3" min="1" max="10"/>
-    <col width="13" customWidth="1" style="3" min="11" max="11"/>
-    <col width="14" customWidth="1" style="3" min="12" max="12"/>
-    <col width="12" customWidth="1" style="3" min="13" max="13"/>
-    <col width="9" customWidth="1" style="3" min="14" max="16384"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Class_Name</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Item_Code</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Size1_From</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Size1_To</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Size2_From</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Size2_To</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Mat_Code</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Mat_Class</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Rating</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Facing</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Flange_Type</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Dim_Standard</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>AA1</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>A105</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>CL150</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>RF</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr">
-        <is>
-          <t>SW</t>
-        </is>
-      </c>
-      <c r="L2" s="3" t="inlineStr">
-        <is>
-          <t>ASME B16.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>AA1</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>A105</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>CL150</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>RF</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>WN</t>
-        </is>
-      </c>
-      <c r="L3" s="3" t="inlineStr">
-        <is>
-          <t>ASME B16.5</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Replace per-class Size Range with Global Size Selection + From/To
Move size availability into a template-wide Size_Selection sheet (NPS↔DN 1:1 table) and per-class Size_From/Size_To columns on Class_Define. Reducing/Branch matrix editors switch to a single Size_From/Size_To range per table; the Size Range wizard tab is removed. NPS/DN catalog extended to NPS 100 / DN 2500.
</commit_message>
<xml_diff>
--- a/tests/input/2604081338_Sample-Class-Input/Class_Define_Template.xlsx
+++ b/tests/input/2604081338_Sample-Class-Input/Class_Define_Template.xlsx
@@ -18,6 +18,7 @@
     <sheet name="Flange_Group" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Gasket_Group" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Valve" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Size_Selection" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Branch_Table'!$A$1:$E$125</definedName>
@@ -89,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -102,6 +103,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -949,13 +953,922 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C63"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>DN</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Use</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>0.125</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>0.375</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1.25</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>450</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>550</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>600</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>650</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>700</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>750</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>800</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>900</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1100</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1250</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1350</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>1400</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1450</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1500</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>1550</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>1600</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>1650</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>1700</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1750</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1850</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>1900</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>1950</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2050</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2100</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2150</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2200</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2250</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2300</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>94</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2350</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>96</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2400</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>98</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2450</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2500</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:T2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="13" customWidth="1" style="3" min="1" max="1"/>
@@ -1067,6 +1980,16 @@
           <t>Remarks</t>
         </is>
       </c>
+      <c r="S1" s="5" t="inlineStr">
+        <is>
+          <t>Size_From</t>
+        </is>
+      </c>
+      <c r="T1" s="5" t="inlineStr">
+        <is>
+          <t>Size_To</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="B2" s="3" t="inlineStr">
@@ -1097,6 +2020,16 @@
       <c r="O2" s="3" t="inlineStr">
         <is>
           <t>RT1</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>24</t>
         </is>
       </c>
     </row>
@@ -1328,7 +2261,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E125"/>
+  <dimension ref="A1:H125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="12" customWidth="1" style="3" min="1" max="5"/>
@@ -1361,6 +2294,21 @@
           <t>Remarks</t>
         </is>
       </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Nominal_Size_System</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Size_From</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Size_To</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -1383,6 +2331,21 @@
           <t>T</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -1405,6 +2368,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1427,6 +2405,21 @@
           <t>T</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1449,6 +2442,21 @@
           <t>R</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -1471,6 +2479,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1493,6 +2516,21 @@
           <t>T</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -1515,6 +2553,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1537,6 +2590,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1559,6 +2627,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1581,6 +2664,21 @@
           <t>T</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1603,6 +2701,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1625,6 +2738,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1647,6 +2775,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1669,6 +2812,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -1691,6 +2849,21 @@
           <t>T</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1713,6 +2886,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -1735,6 +2923,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -1757,6 +2960,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1779,6 +2997,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -1801,6 +3034,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1823,6 +3071,21 @@
           <t>T</t>
         </is>
       </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -1845,6 +3108,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -1867,6 +3145,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -1889,6 +3182,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -1911,6 +3219,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -1933,6 +3256,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -1955,6 +3293,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -1977,6 +3330,21 @@
           <t>T</t>
         </is>
       </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -1999,6 +3367,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -2021,6 +3404,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -2043,6 +3441,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -2065,6 +3478,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -2087,6 +3515,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -2109,6 +3552,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -2131,6 +3589,21 @@
           <t>T</t>
         </is>
       </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -2153,6 +3626,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -2175,6 +3663,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -2197,6 +3700,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -2219,6 +3737,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -2241,6 +3774,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
@@ -2263,6 +3811,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -2285,6 +3848,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -2307,6 +3885,21 @@
           <t>T</t>
         </is>
       </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -2329,6 +3922,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
@@ -2351,6 +3959,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -2373,6 +3996,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
@@ -2395,6 +4033,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -2417,6 +4070,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
@@ -2439,6 +4107,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -2461,6 +4144,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
@@ -2483,6 +4181,21 @@
           <t>T</t>
         </is>
       </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
@@ -2505,6 +4218,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
@@ -2527,6 +4255,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -2549,6 +4292,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
@@ -2571,6 +4329,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
@@ -2593,6 +4366,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
@@ -2615,6 +4403,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -2637,6 +4440,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
@@ -2659,6 +4477,21 @@
           <t>T</t>
         </is>
       </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
@@ -2681,6 +4514,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
@@ -2703,6 +4551,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
@@ -2725,6 +4588,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
@@ -2747,6 +4625,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
@@ -2769,6 +4662,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
@@ -2791,6 +4699,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
@@ -2813,6 +4736,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
@@ -2835,6 +4773,21 @@
           <t>T</t>
         </is>
       </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
@@ -2857,6 +4810,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
@@ -2879,6 +4847,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
@@ -2901,6 +4884,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
@@ -2923,6 +4921,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
@@ -2945,6 +4958,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
@@ -2967,6 +4995,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
@@ -2989,6 +5032,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
@@ -3011,6 +5069,21 @@
           <t>T</t>
         </is>
       </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
@@ -3033,6 +5106,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
@@ -3055,6 +5143,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
@@ -3077,6 +5180,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
@@ -3099,6 +5217,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
@@ -3121,6 +5254,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
@@ -3143,6 +5291,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
@@ -3165,6 +5328,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
@@ -3187,6 +5365,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
@@ -3209,6 +5402,21 @@
           <t>T</t>
         </is>
       </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
@@ -3231,6 +5439,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
@@ -3253,6 +5476,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
@@ -3275,6 +5513,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
@@ -3297,6 +5550,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
@@ -3319,6 +5587,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
@@ -3341,6 +5624,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
@@ -3363,6 +5661,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
@@ -3385,6 +5698,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
@@ -3407,6 +5735,21 @@
           <t>T</t>
         </is>
       </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
@@ -3429,6 +5772,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
@@ -3451,6 +5809,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
@@ -3473,6 +5846,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
@@ -3495,6 +5883,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
@@ -3517,6 +5920,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
@@ -3539,6 +5957,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
@@ -3561,6 +5994,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
@@ -3583,6 +6031,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
@@ -3605,6 +6068,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
@@ -3627,6 +6105,21 @@
           <t>T</t>
         </is>
       </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
@@ -3649,6 +6142,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
@@ -3671,6 +6179,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
@@ -3693,6 +6216,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
@@ -3715,6 +6253,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
@@ -3737,6 +6290,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
@@ -3759,6 +6327,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
@@ -3781,6 +6364,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
@@ -3803,6 +6401,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
@@ -3825,6 +6438,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="3" t="inlineStr">
@@ -3847,6 +6475,21 @@
           <t>T</t>
         </is>
       </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
@@ -3869,6 +6512,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="3" t="inlineStr">
@@ -3891,6 +6549,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
@@ -3913,6 +6586,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="3" t="inlineStr">
@@ -3935,6 +6623,21 @@
           <t>TH</t>
         </is>
       </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
@@ -3957,6 +6660,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
@@ -3979,6 +6697,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
@@ -4001,6 +6734,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
@@ -4023,6 +6771,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
@@ -4045,6 +6808,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
@@ -4067,6 +6845,21 @@
           <t>RT</t>
         </is>
       </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
@@ -4087,6 +6880,21 @@
       <c r="D125" s="3" t="inlineStr">
         <is>
           <t>T</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>24</t>
         </is>
       </c>
     </row>
@@ -4102,7 +6910,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="12" customWidth="1" style="3" min="1" max="5"/>
@@ -4135,6 +6943,21 @@
           <t>Remarks</t>
         </is>
       </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Nominal_Size_System</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Size_From</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Size_To</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -4157,6 +6980,21 @@
           <t>SN</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -4179,6 +7017,21 @@
           <t>SN</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -4201,6 +7054,21 @@
           <t>SN</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -4223,6 +7091,21 @@
           <t>SN</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -4245,6 +7128,21 @@
           <t>SN</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -4267,6 +7165,21 @@
           <t>SN</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -4289,6 +7202,21 @@
           <t>SN</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -4311,6 +7239,21 @@
           <t>SN</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -4333,6 +7276,21 @@
           <t>SN</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -4355,6 +7313,21 @@
           <t>SN</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -4377,6 +7350,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -4399,6 +7387,21 @@
           <t>SN</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -4421,6 +7424,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -4443,6 +7461,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -4465,6 +7498,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -4487,6 +7535,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -4509,6 +7572,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -4531,6 +7609,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -4553,6 +7646,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -4575,6 +7683,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -4597,6 +7720,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -4619,6 +7757,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -4641,6 +7794,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -4663,6 +7831,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -4685,6 +7868,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -4707,6 +7905,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -4729,6 +7942,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -4751,6 +7979,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -4773,6 +8016,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -4795,6 +8053,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -4817,6 +8090,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -4839,6 +8127,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -4861,6 +8164,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -4883,6 +8201,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -4905,6 +8238,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -4927,6 +8275,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -4949,6 +8312,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -4971,6 +8349,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -4993,6 +8386,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -5015,6 +8423,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
@@ -5037,6 +8460,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -5059,6 +8497,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -5081,6 +8534,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -5103,6 +8571,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
@@ -5125,6 +8608,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -5147,6 +8645,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
@@ -5169,6 +8682,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -5191,6 +8719,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
@@ -5213,6 +8756,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -5235,6 +8793,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
@@ -5257,6 +8830,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
@@ -5279,6 +8867,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
@@ -5301,6 +8904,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -5323,6 +8941,21 @@
           <t>RD</t>
         </is>
       </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
@@ -5343,6 +8976,21 @@
       <c r="D56" s="3" t="inlineStr">
         <is>
           <t>RD</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>24</t>
         </is>
       </c>
     </row>

</xml_diff>